<commit_message>
chore(preview): MSFT outputs regeneres
</commit_message>
<xml_diff>
--- a/preview/MSFT/MSFT_financials.xlsx
+++ b/preview/MSFT/MSFT_financials.xlsx
@@ -13642,7 +13642,7 @@
       </c>
       <c r="D120" s="239" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="E120" s="240" t="n"/>
@@ -24216,7 +24216,7 @@
         <v>253.5</v>
       </c>
       <c r="E9" s="589" t="n">
-        <v>3823961.9</v>
+        <v>3745270.99</v>
       </c>
       <c r="F9" s="589" t="n">
         <v>435617.01</v>
@@ -24256,7 +24256,7 @@
         <v>303.93</v>
       </c>
       <c r="E10" s="589" t="n">
-        <v>3540945.99</v>
+        <v>3616794.21</v>
       </c>
       <c r="F10" s="589" t="n">
         <v>402836</v>
@@ -24296,7 +24296,7 @@
         <v>143.17</v>
       </c>
       <c r="E11" s="589" t="n">
-        <v>547122.74</v>
+        <v>540306.51</v>
       </c>
       <c r="F11" s="589" t="n">
         <v>64076</v>
@@ -24336,7 +24336,7 @@
         <v>145.22</v>
       </c>
       <c r="E12" s="589" t="n">
-        <v>172275.55</v>
+        <v>167978.93</v>
       </c>
       <c r="F12" s="589" t="n">
         <v>36800</v>
@@ -24373,10 +24373,10 @@
         </is>
       </c>
       <c r="D13" s="591" t="n">
-        <v>182.99</v>
+        <v>182.96</v>
       </c>
       <c r="E13" s="592" t="n">
-        <v>178928.7</v>
+        <v>177018.08</v>
       </c>
       <c r="F13" s="592" t="n">
         <v>41525</v>

</xml_diff>